<commit_message>
Enhance JISResult with comprehensive validation checks for solution constraints, ensuring compliance with business rules. Integrate logging for issue reporting during checks. Update JISCPModel to correct constraint logic for pallet assignments. Add 'loguru' dependency for improved logging capabilities.
</commit_message>
<xml_diff>
--- a/result/result_sample_input.xlsx
+++ b/result/result_sample_input.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t>供应商</t>
   </si>
@@ -28,7 +28,13 @@
     <t>任务令</t>
   </si>
   <si>
-    <t>满足量</t>
+    <t>线体</t>
+  </si>
+  <si>
+    <t>货位</t>
+  </si>
+  <si>
+    <t>任务令满足量</t>
   </si>
   <si>
     <t>包规</t>
@@ -37,27 +43,21 @@
     <t>装载板数</t>
   </si>
   <si>
+    <t>装载量</t>
+  </si>
+  <si>
     <t>总装载板数</t>
   </si>
   <si>
     <t>车规</t>
   </si>
   <si>
+    <t>装载率</t>
+  </si>
+  <si>
     <t>到达时间</t>
   </si>
   <si>
-    <t>装载率</t>
-  </si>
-  <si>
-    <t>s_group</t>
-  </si>
-  <si>
-    <t>sv_group</t>
-  </si>
-  <si>
-    <t>svi_group</t>
-  </si>
-  <si>
     <t>supplier1</t>
   </si>
   <si>
@@ -73,13 +73,19 @@
     <t>mfg_order1</t>
   </si>
   <si>
+    <t>line1</t>
+  </si>
+  <si>
+    <t>loc1</t>
+  </si>
+  <si>
+    <t>11.11%</t>
+  </si>
+  <si>
+    <t>9.09%</t>
+  </si>
+  <si>
     <t>2026-06-09 21:00:00</t>
-  </si>
-  <si>
-    <t>11.11%</t>
-  </si>
-  <si>
-    <t>9.09%</t>
   </si>
 </sst>
 </file>
@@ -471,35 +477,35 @@
       <c r="D2" t="s">
         <v>18</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2">
         <v>60</v>
       </c>
-      <c r="F2">
+      <c r="H2">
         <v>30</v>
       </c>
-      <c r="G2">
+      <c r="I2">
         <v>2</v>
       </c>
-      <c r="H2">
+      <c r="J2">
+        <v>60</v>
+      </c>
+      <c r="K2">
         <v>2</v>
       </c>
-      <c r="I2">
+      <c r="L2">
         <v>18</v>
       </c>
-      <c r="J2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
+      <c r="M2" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -515,35 +521,35 @@
       <c r="D3" t="s">
         <v>18</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3">
         <v>40</v>
       </c>
-      <c r="F3">
+      <c r="H3">
         <v>30</v>
       </c>
-      <c r="G3">
+      <c r="I3">
         <v>2</v>
       </c>
-      <c r="H3">
+      <c r="J3">
+        <v>60</v>
+      </c>
+      <c r="K3">
         <v>2</v>
       </c>
-      <c r="I3">
+      <c r="L3">
         <v>22</v>
       </c>
-      <c r="J3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-      <c r="N3">
-        <v>1</v>
+      <c r="M3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update result_sample_input.xlsx to reflect recent changes in data structure and improve compatibility with JISResult output. This update enhances the overall data representation in Excel format.
</commit_message>
<xml_diff>
--- a/result/result_sample_input.xlsx
+++ b/result/result_sample_input.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
   <si>
     <t>供应商</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>9.09%</t>
+  </si>
+  <si>
+    <t>2026-06-09 20:00:00</t>
   </si>
   <si>
     <t>2026-06-09 21:00:00</t>
@@ -484,7 +487,7 @@
         <v>20</v>
       </c>
       <c r="G2">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H2">
         <v>30</v>
@@ -528,7 +531,7 @@
         <v>20</v>
       </c>
       <c r="G3">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H3">
         <v>30</v>
@@ -549,7 +552,7 @@
         <v>22</v>
       </c>
       <c r="N3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add FastAPI and related dependencies for web application development. Introduce new web module with app structure, including file upload handling and parameter configuration for optimization. Implement frontend with HTML, CSS, and JavaScript for user interaction. Enhance JISData with error handling for arrival time selection.
</commit_message>
<xml_diff>
--- a/result/result_sample_input.xlsx
+++ b/result/result_sample_input.xlsx
@@ -487,7 +487,7 @@
         <v>20</v>
       </c>
       <c r="G2">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H2">
         <v>30</v>
@@ -531,7 +531,7 @@
         <v>20</v>
       </c>
       <c r="G3">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H3">
         <v>30</v>

</xml_diff>